<commit_message>
done with TOKZ_DZT. initial tested
</commit_message>
<xml_diff>
--- a/mode_docx_gen/pmi_lodzt/part/lvalh/CALH1.xlsx
+++ b/mode_docx_gen/pmi_lodzt/part/lvalh/CALH1.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\www5\mode_docx_gen\pmi_dzt\part\lvalh\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\www5\mode_docx_gen\pmi_lodzt\part\lvalh\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="90">
   <si>
     <t>Категория (group)</t>
   </si>
@@ -148,12 +148,15 @@
     <t>Hash</t>
   </si>
   <si>
-    <t>Пред. сигн.</t>
+    <t>DZT2_LVALH</t>
   </si>
   <si>
     <t>Контроль сигнала &lt;&lt;ТЗ сигн&gt;&gt;</t>
   </si>
   <si>
+    <t>Контр_ТЗ_сигн</t>
+  </si>
+  <si>
     <t>Пуск</t>
   </si>
   <si>
@@ -172,6 +175,9 @@
     <t>Контроль сигнала &lt;&lt;ГЗ сигн&gt;&gt;</t>
   </si>
   <si>
+    <t>Контр_ГЗ_сигн</t>
+  </si>
+  <si>
     <t>Контроль сигнала &lt;&lt;Низ.изол. ТЗ&gt;&gt;</t>
   </si>
   <si>
@@ -196,18 +202,30 @@
     <t>Контроль сигнала &lt;&lt;Низ.изол. ГЗ&gt;&gt;</t>
   </si>
   <si>
+    <t>Контр_ТС_сигн</t>
+  </si>
+  <si>
     <t>Контроль сигнала &lt;&lt;ТС сигн&gt;&gt;</t>
   </si>
   <si>
+    <t>Контр_ОТ_сигн</t>
+  </si>
+  <si>
     <t>Контроль сигнала &lt;&lt;ОТ сигн&gt;&gt;</t>
   </si>
   <si>
+    <t>Контр_ОТ_НН_сигн</t>
+  </si>
+  <si>
     <t>Контроль сигнала &lt;&lt;ОТ НН сигн&gt;&gt;</t>
   </si>
   <si>
     <t>Контроль сигнала &lt;&lt;Внеш. откл&gt;&gt;</t>
   </si>
   <si>
+    <t>Контр_Внеш_откл</t>
+  </si>
+  <si>
     <t>SGF9</t>
   </si>
   <si>
@@ -217,75 +235,45 @@
     <t>Контроль сигнала &lt;&lt;Вых. цепи разобраны&gt;&gt;</t>
   </si>
   <si>
+    <t>Контр_БИ_выведены</t>
+  </si>
+  <si>
     <t>Контроль сигнала &lt;&lt;БИ выведены&gt;&gt;</t>
   </si>
   <si>
     <t>SGF11</t>
   </si>
   <si>
-    <t>Контроль сигнала &lt;&lt;Прев. вр. пер. КА&gt;&gt;</t>
-  </si>
-  <si>
     <t>SGF12</t>
   </si>
   <si>
+    <t>Контроль сигнала &lt;&lt;ГЗ заблокирована&gt;&gt;</t>
+  </si>
+  <si>
+    <t>Контр_ГЗ_блок</t>
+  </si>
+  <si>
+    <t>Контроль сигнала &lt;&lt;ТЗ заблокирована&gt;&gt;</t>
+  </si>
+  <si>
+    <t>Контр_ТЗ_блок</t>
+  </si>
+  <si>
+    <t>DZT_LVCALH_UIRZ</t>
+  </si>
+  <si>
+    <t>Контр_Низ_изол_ТЗ</t>
+  </si>
+  <si>
+    <t>Контр_Низ_изол_ГЗ</t>
+  </si>
+  <si>
+    <t>Контр_Вых_цеп_разоб</t>
+  </si>
+  <si>
     <t>SGF13</t>
   </si>
   <si>
-    <t>T_LVALH</t>
-  </si>
-  <si>
-    <t>Контроль сигнала &lt;&lt;ГЗ заблокирована&gt;&gt;</t>
-  </si>
-  <si>
-    <t>Контр_ГЗ_блок</t>
-  </si>
-  <si>
-    <t>Контроль сигнала &lt;&lt;ТЗ заблокирована&gt;&gt;</t>
-  </si>
-  <si>
-    <t>Контр_ТЗ_блок</t>
-  </si>
-  <si>
-    <t>SGF14</t>
-  </si>
-  <si>
-    <t>Контр_ТЗ_сигн</t>
-  </si>
-  <si>
-    <t>Контр_ГЗ_сигн</t>
-  </si>
-  <si>
-    <t>Контр_Низ_изол_ТЗ</t>
-  </si>
-  <si>
-    <t>Контр_Низ_изол_ГЗ</t>
-  </si>
-  <si>
-    <t>Контр_ТС_сигн</t>
-  </si>
-  <si>
-    <t>Контр_ОТ_сигн</t>
-  </si>
-  <si>
-    <t>Контр_ОТ_НН_сигн</t>
-  </si>
-  <si>
-    <t>Контр_Внеш_откл</t>
-  </si>
-  <si>
-    <t>Контр_Вых_цеп_разоб</t>
-  </si>
-  <si>
-    <t>Контр_БИ_выведены</t>
-  </si>
-  <si>
-    <t>Контр_Вр_пркл_КА</t>
-  </si>
-  <si>
-    <t>T_LVCALH</t>
-  </si>
-  <si>
     <t>Контроль общего внешнего сигнала</t>
   </si>
   <si>
@@ -295,10 +283,10 @@
     <t>DescriptionFunc</t>
   </si>
   <si>
+    <t>WeightFunc</t>
+  </si>
+  <si>
     <t>Предупредительная сигнализация</t>
-  </si>
-  <si>
-    <t>WeightFunc</t>
   </si>
   <si>
     <t>alias</t>
@@ -320,6 +308,8 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
   </fonts>
   <fills count="6">
@@ -694,18 +684,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AE17"/>
+  <dimension ref="A1:AE16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="3"/>
     <col min="3" max="3" width="48.28515625" style="3" customWidth="1"/>
-    <col min="4" max="4" width="23.85546875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="3" customWidth="1"/>
     <col min="5" max="5" width="12.28515625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="41.5703125" style="3" customWidth="1"/>
+    <col min="6" max="6" width="20" style="3" customWidth="1"/>
     <col min="7" max="7" width="9.140625" style="3"/>
     <col min="8" max="8" width="7.140625" style="3" customWidth="1"/>
     <col min="9" max="12" width="9.140625" style="3"/>
-    <col min="13" max="13" width="15.5703125" style="3" customWidth="1"/>
+    <col min="13" max="13" width="18.85546875" style="3" customWidth="1"/>
     <col min="14" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
@@ -801,7 +791,7 @@
         <v>29</v>
       </c>
       <c r="AE1" s="3" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.25">
@@ -809,13 +799,13 @@
         <v>33</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>34</v>
@@ -841,8 +831,8 @@
       <c r="L2" s="3">
         <v>0</v>
       </c>
-      <c r="M2" s="6" t="s">
-        <v>87</v>
+      <c r="M2" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="N2" s="3" t="s">
         <v>31</v>
@@ -901,13 +891,13 @@
         <v>33</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>36</v>
@@ -933,8 +923,8 @@
       <c r="L3" s="3">
         <v>0</v>
       </c>
-      <c r="M3" s="6" t="s">
-        <v>87</v>
+      <c r="M3" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>31</v>
@@ -993,16 +983,16 @@
         <v>33</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>35</v>
@@ -1025,8 +1015,8 @@
       <c r="L4" s="3">
         <v>0</v>
       </c>
-      <c r="M4" s="6" t="s">
-        <v>87</v>
+      <c r="M4" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="N4" s="3" t="s">
         <v>31</v>
@@ -1085,16 +1075,16 @@
         <v>33</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>43</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>76</v>
+        <v>44</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>35</v>
@@ -1117,8 +1107,8 @@
       <c r="L5" s="3">
         <v>0</v>
       </c>
-      <c r="M5" s="6" t="s">
-        <v>87</v>
+      <c r="M5" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="N5" s="3" t="s">
         <v>31</v>
@@ -1177,16 +1167,16 @@
         <v>33</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>35</v>
@@ -1209,8 +1199,8 @@
       <c r="L6" s="5">
         <v>0</v>
       </c>
-      <c r="M6" s="6" t="s">
-        <v>87</v>
+      <c r="M6" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="N6" s="5" t="s">
         <v>31</v>
@@ -1269,16 +1259,16 @@
         <v>33</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>35</v>
@@ -1301,8 +1291,8 @@
       <c r="L7" s="5">
         <v>0</v>
       </c>
-      <c r="M7" s="6" t="s">
-        <v>87</v>
+      <c r="M7" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="N7" s="5" t="s">
         <v>31</v>
@@ -1361,16 +1351,16 @@
         <v>33</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>55</v>
+        <v>60</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>35</v>
@@ -1393,8 +1383,8 @@
       <c r="L8" s="3">
         <v>0</v>
       </c>
-      <c r="M8" s="6" t="s">
-        <v>87</v>
+      <c r="M8" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="N8" s="3" t="s">
         <v>31</v>
@@ -1453,16 +1443,16 @@
         <v>33</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>56</v>
+        <v>62</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>58</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>35</v>
@@ -1485,8 +1475,8 @@
       <c r="L9" s="3">
         <v>0</v>
       </c>
-      <c r="M9" s="6" t="s">
-        <v>87</v>
+      <c r="M9" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="N9" s="3" t="s">
         <v>31</v>
@@ -1545,16 +1535,16 @@
         <v>33</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>68</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>35</v>
@@ -1577,8 +1567,8 @@
       <c r="L10" s="3">
         <v>0</v>
       </c>
-      <c r="M10" s="6" t="s">
-        <v>87</v>
+      <c r="M10" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="N10" s="3" t="s">
         <v>31</v>
@@ -1637,16 +1627,16 @@
         <v>33</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>63</v>
+        <v>67</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>69</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>35</v>
@@ -1669,8 +1659,8 @@
       <c r="L11" s="3">
         <v>0</v>
       </c>
-      <c r="M11" s="6" t="s">
-        <v>87</v>
+      <c r="M11" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="N11" s="3" t="s">
         <v>31</v>
@@ -1729,16 +1719,16 @@
         <v>33</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>66</v>
+        <v>82</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>35</v>
@@ -1761,8 +1751,8 @@
       <c r="L12" s="3">
         <v>0</v>
       </c>
-      <c r="M12" s="6" t="s">
-        <v>87</v>
+      <c r="M12" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="N12" s="3" t="s">
         <v>31</v>
@@ -1821,16 +1811,16 @@
         <v>33</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>68</v>
+        <v>71</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>74</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>35</v>
@@ -1853,8 +1843,8 @@
       <c r="L13" s="3">
         <v>0</v>
       </c>
-      <c r="M13" s="6" t="s">
-        <v>87</v>
+      <c r="M13" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="N13" s="3" t="s">
         <v>31</v>
@@ -1908,187 +1898,187 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:31" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="F14" s="3" t="s">
+      <c r="B14" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="F14" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="G14" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="H14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I14" s="3">
-        <v>0</v>
-      </c>
-      <c r="J14" s="3">
-        <v>1</v>
-      </c>
-      <c r="K14" s="3">
-        <v>1</v>
-      </c>
-      <c r="L14" s="3">
-        <v>0</v>
-      </c>
-      <c r="M14" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="N14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="O14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="P14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="R14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="S14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="T14" s="3">
-        <v>0</v>
-      </c>
-      <c r="U14" s="3">
-        <v>0</v>
-      </c>
-      <c r="V14" s="3">
-        <v>0</v>
-      </c>
-      <c r="W14" s="3">
-        <v>0</v>
-      </c>
-      <c r="X14" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y14" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z14" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="AB14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="AC14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="AD14" s="3" t="s">
+      <c r="H14" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="I14" s="7">
+        <v>0</v>
+      </c>
+      <c r="J14" s="7">
+        <v>1</v>
+      </c>
+      <c r="K14" s="7">
+        <v>1</v>
+      </c>
+      <c r="L14" s="7">
+        <v>0</v>
+      </c>
+      <c r="M14" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="N14" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="O14" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="P14" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q14" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="R14" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="S14" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="T14" s="7">
+        <v>0</v>
+      </c>
+      <c r="U14" s="7">
+        <v>0</v>
+      </c>
+      <c r="V14" s="7">
+        <v>0</v>
+      </c>
+      <c r="W14" s="7">
+        <v>0</v>
+      </c>
+      <c r="X14" s="7">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="7">
+        <v>0</v>
+      </c>
+      <c r="Z14" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="AB14" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="AC14" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD14" s="7" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:31" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="G15" s="7" t="s">
+    <row r="15" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="H15" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="I15" s="7">
-        <v>0</v>
-      </c>
-      <c r="J15" s="7">
-        <v>1</v>
-      </c>
-      <c r="K15" s="7">
-        <v>1</v>
-      </c>
-      <c r="L15" s="7">
-        <v>0</v>
-      </c>
-      <c r="M15" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="N15" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="O15" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="P15" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q15" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="R15" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="S15" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="T15" s="7">
-        <v>0</v>
-      </c>
-      <c r="U15" s="7">
-        <v>0</v>
-      </c>
-      <c r="V15" s="7">
-        <v>0</v>
-      </c>
-      <c r="W15" s="7">
-        <v>0</v>
-      </c>
-      <c r="X15" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y15" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA15" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="AB15" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="AC15" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="AD15" s="7" t="s">
+      <c r="H15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="M15" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="N15" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="O15" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="P15" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q15" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="R15" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="S15" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="T15" s="4">
+        <v>0</v>
+      </c>
+      <c r="U15" s="4">
+        <v>1</v>
+      </c>
+      <c r="V15" s="4">
+        <v>0</v>
+      </c>
+      <c r="W15" s="4">
+        <v>1</v>
+      </c>
+      <c r="X15" s="4">
+        <v>1</v>
+      </c>
+      <c r="Y15" s="4">
+        <v>1</v>
+      </c>
+      <c r="Z15" s="4">
+        <v>1</v>
+      </c>
+      <c r="AA15" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="AB15" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="AC15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD15" s="2" t="s">
         <v>31</v>
       </c>
     </row>
@@ -2097,16 +2087,16 @@
         <v>30</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>48</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>31</v>
@@ -2129,8 +2119,8 @@
       <c r="L16" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="M16" s="6" t="s">
-        <v>87</v>
+      <c r="M16" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="N16" s="3" t="s">
         <v>31</v>
@@ -2181,98 +2171,6 @@
         <v>31</v>
       </c>
       <c r="AD16" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="L17" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="M17" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="N17" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="O17" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="P17" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q17" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="R17" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="S17" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="T17" s="4">
-        <v>0</v>
-      </c>
-      <c r="U17" s="4">
-        <v>1</v>
-      </c>
-      <c r="V17" s="4">
-        <v>0</v>
-      </c>
-      <c r="W17" s="4">
-        <v>1</v>
-      </c>
-      <c r="X17" s="4">
-        <v>1</v>
-      </c>
-      <c r="Y17" s="4">
-        <v>1</v>
-      </c>
-      <c r="Z17" s="4">
-        <v>1</v>
-      </c>
-      <c r="AA17" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="AB17" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="AC17" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="AD17" s="2" t="s">
         <v>31</v>
       </c>
     </row>
@@ -2287,7 +2185,8 @@
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.140625" customWidth="1"/>
+    <col min="1" max="1" width="27.85546875" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -2303,7 +2202,7 @@
         <v>39</v>
       </c>
       <c r="B2" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -2311,7 +2210,7 @@
         <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -2321,15 +2220,15 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B5" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B6">
         <v>10</v>

</xml_diff>